<commit_message>
feat(ui): highlight low balances and refresh onboarding sample
</commit_message>
<xml_diff>
--- a/public/sample-onboarding-import-v2.xlsx
+++ b/public/sample-onboarding-import-v2.xlsx
@@ -480,7 +480,7 @@
         <v>CashWallet</v>
       </c>
       <c r="C5">
-        <v>2500</v>
+        <v>3600</v>
       </c>
       <c r="D5" t="str">
         <v>Wallet</v>
@@ -1653,7 +1653,7 @@
         <v>Transfer</v>
       </c>
       <c r="C10">
-        <v>1500</v>
+        <v>1700</v>
       </c>
       <c r="D10" t="str">
         <v>2025-10-06</v>
@@ -2325,7 +2325,7 @@
         <v>Transfer</v>
       </c>
       <c r="C31">
-        <v>1500</v>
+        <v>1800</v>
       </c>
       <c r="D31" t="str">
         <v>2025-11-06</v>
@@ -3029,7 +3029,7 @@
         <v>Transfer</v>
       </c>
       <c r="C53">
-        <v>1800</v>
+        <v>1900</v>
       </c>
       <c r="D53" t="str">
         <v>2025-12-06</v>
@@ -3765,7 +3765,7 @@
         <v>Transfer</v>
       </c>
       <c r="C76">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="D76" t="str">
         <v>2026-01-06</v>
@@ -4437,7 +4437,7 @@
         <v>Transfer</v>
       </c>
       <c r="C97">
-        <v>1800</v>
+        <v>2100</v>
       </c>
       <c r="D97" t="str">
         <v>2026-02-06</v>
@@ -5173,7 +5173,7 @@
         <v>Transfer</v>
       </c>
       <c r="C120">
-        <v>1700</v>
+        <v>2250</v>
       </c>
       <c r="D120" t="str">
         <v>2026-03-06</v>

</xml_diff>